<commit_message>
투자 대시보드 2026-10-01 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-09-30.xlsx
+++ b/technicals/exports/2026-09-30.xlsx
@@ -135,11 +135,6 @@
           <ns0:t/>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>엣지부터 클라우드까지 IT 및 기업용 제품·솔루션·서비스를 제공하는 글로벌 기업.</ns0:t>
-        </ns0:is>
-      </ns0:c>
       <ns0:c r="G2">
         <ns0:v>63.88999938964844</ns0:v>
       </ns0:c>
@@ -187,11 +182,6 @@
           <ns0:t>https://finance.yahoo.com/technology/ai/articles/hpe-shares-jump-1-2-180808900.html</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="T2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>https://finviz.com/quote.ashx?t=HPE</ns0:t>
-        </ns0:is>
-      </ns0:c>
     </ns0:row>
     <ns0:row r="3">
       <ns0:c r="A3" t="inlineStr">
@@ -221,7 +211,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>미충족 의료 수요를 위한 항체 의약품을 개발하며, 비호르몬성 ABCL635는 혈관운동 증상 대상 임상 2상 중.</ns0:t>
+          <ns0:t>미충족 의료 수요를 위한 항체 치료제 개발사. 비호르몬성 ABCL635는 혈관운동 증상 임상 2상 중.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
@@ -263,7 +253,7 @@
       </ns0:c>
       <ns0:c r="R3" t="inlineStr">
         <ns0:is>
-          <ns0:t>ABCL을 포함한 종목들의 주가 급등과 52주 최고치 기록을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>ABCL 등 종목의 52주 신고가 기록과 급등 배경을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S3" t="inlineStr">
@@ -305,7 +295,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국 뷰티·개인관리 브랜드에 전략, 마케팅, 전 채널 판매, 고객 서비스 및 물류 등 브랜드 관리 제공.</ns0:t>
+          <ns0:t>중국 뷰티·개인관리 브랜드에 전략·마케팅·전 채널 판매·고객 서비스·물류 등 브랜드 관리 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -423,7 +413,7 @@
       </ns0:c>
       <ns0:c r="R5" t="inlineStr">
         <ns0:is>
-          <ns0:t>임상시험 업데이트와 신규 자금 조달 이후 아제너스 주식의 적정가치 평가가 높아졌다는 보도다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>임상 진행 소식과 신규 자금 조달 이후 아제너스 주식의 적정가치 평가 상향 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S5" t="inlineStr">
@@ -507,7 +497,7 @@
       </ns0:c>
       <ns0:c r="R6" t="inlineStr">
         <ns0:is>
-          <ns0:t>올해 앳코어 주가가 산업재 동종 기업보다 높은 성과를 내는지 비교. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>올해 주가 성과가 산업재 동종 기업을 앞서는지 비교하는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S6" t="inlineStr">
@@ -591,7 +581,7 @@
       </ns0:c>
       <ns0:c r="R7" t="inlineStr">
         <ns0:is>
-          <ns0:t>AI 관련 반도체 수요를 전망하며 4분기 매출 반등을 목표로 한다는 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>AI 관련 반도체 수요 확대를 전망하며 4분기 매출 반등을 목표로 한다는 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S7" t="inlineStr">
@@ -633,7 +623,7 @@
       </ns0:c>
       <ns0:c r="F8" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 기업·비영리단체·기업가에게 은행 상품과 서비스를 제공하는 Capital Bank의 지주회사.</ns0:t>
+          <ns0:t>미국 기업·비영리단체·기업가에게 은행 서비스를 제공하는 Capital Bank의 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G8">
@@ -675,7 +665,7 @@
       </ns0:c>
       <ns0:c r="R8" t="inlineStr">
         <ns0:is>
-          <ns0:t>매수 등급 상향 소식과 함께 가치투자 관점의 매수 적절성 및 저평가 여부를 다룬 분석. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>투자의견 매수 상향과 함께 가치투자 관점의 매수 적합성 및 저평가 여부를 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S8" t="inlineStr">
@@ -717,7 +707,7 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>이식 환자의 치료 결과와 장기 건강 개선을 위한 신장·심장 이식 검사 솔루션 등을 제공하는 기업.</ns0:t>
+          <ns0:t>이식 환자의 치료 결과와 장기 건강 개선을 위한 신장·심장 이식 검사 솔루션 제공 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9">
@@ -801,7 +791,7 @@
       </ns0:c>
       <ns0:c r="F10" t="inlineStr">
         <ns0:is>
-          <ns0:t>Citizens and Farmers Bank의 은행지주사로 개인·기업 금융, 주택담보대출 및 소비자금융 제공.</ns0:t>
+          <ns0:t>Citizens and Farmers Bank의 지주사로 개인·기업 금융, 주택담보대출·소비자금융 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G10">
@@ -927,7 +917,7 @@
       </ns0:c>
       <ns0:c r="R11" t="inlineStr">
         <ns0:is>
-          <ns0:t>주가 2% 상승 보도와 변동성 대비 보상 분석, 팔로알토 네트웍스와의 투자 비교. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>주가 2% 상승 보도와 변동성 대비 수익 평가, 팔로알토네트웍스와의 투자 비교 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S11" t="inlineStr">
@@ -969,7 +959,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>한국·미국 등에서 캐주얼 게임과 모바일 앱을 개발·배급하며 소셜 카지노와 iGaming 사업 운영.</ns0:t>
+          <ns0:t>한국·미국 등에서 캐주얼 게임·모바일 앱을 개발·배급하며 소셜 카지노와 iGaming 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1011,7 +1001,7 @@
       </ns0:c>
       <ns0:c r="R12" t="inlineStr">
         <ns0:is>
-          <ns0:t>인수 제안이 미해결 상태인 가운데 이익이 급증했다는 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>이익 급증과 아직 결론 나지 않은 인수 제안을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S12" t="inlineStr">
@@ -1053,7 +1043,7 @@
       </ns0:c>
       <ns0:c r="F13" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 난치성 암 치료제를 발굴·개발·상용화하며 진행성 신세포암 치료제 CABOMETYX를 제공.</ns0:t>
+          <ns0:t>미국에서 난치성 암 치료제를 발굴·개발·상용화하며 진행성 신세포암 치료제 CABOMETYX 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G13">
@@ -1095,7 +1085,7 @@
       </ns0:c>
       <ns0:c r="R13" t="inlineStr">
         <ns0:is>
-          <ns0:t>잔잘린티닙의 FDA 지연이 성장 계획에 영향을 미칠 가능성을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>잔잘린티닙의 FDA 절차 지연이 성장 계획에 미칠 영향을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S13" t="inlineStr">
@@ -1216,7 +1206,7 @@
       </ns0:c>
       <ns0:c r="F15" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 다른 기업과의 합병·인수 등 사업결합을 추진하는 기업.</ns0:t>
+          <ns0:t>주요 영업활동 없이 다른 기업과 합병·인수 등 사업결합을 추진하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G15">
@@ -1334,7 +1324,7 @@
       </ns0:c>
       <ns0:c r="R16" t="inlineStr">
         <ns0:is>
-          <ns0:t>올해 포슬 그룹과 소매·도매 업종 주식의 성과를 비교한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>올해 포실그룹과 소매·도매 업종의 주가 성과를 비교하는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S16" t="inlineStr">
@@ -1376,7 +1366,7 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>덴마크 바이오기업으로 암 등 질환 치료용 항체 의약품을 개발하며 EPKINLY·TEPKINLY를 판매한다.</ns0:t>
+          <ns0:t>암 등 질환 치료용 항체 의약품을 개발하고 EPKINLY·TEPKINLY를 판매하는 덴마크 바이오기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17">
@@ -1460,7 +1450,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>다중암 조기검사 기업으로, 50세 초과 무증상자를 위한 암 선별검사 Galleri 등을 제공.</ns0:t>
+          <ns0:t>다중암 조기검사 기업으로 50세 초과 무증상자 대상 암 선별검사 Galleri 등을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1499,7 +1489,7 @@
       </ns0:c>
       <ns0:c r="R18" t="inlineStr">
         <ns0:is>
-          <ns0:t>6개월간 180%, 주간 약 70% 및 55%의 주가 상승을 각각 다룬 기사들이 추가 상승 여력과 관전 요소 조명. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>6개월간 180%, 주간 약 70% 및 55% 주가 급등을 각각 다루며 추가 상승 가능성과 향후 관전 포인트 제시. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S18" t="inlineStr">
@@ -1583,7 +1573,7 @@
       </ns0:c>
       <ns0:c r="R19" t="inlineStr">
         <ns0:is>
-          <ns0:t>Torm 지분을 19.85%로 확대한 뒤 주가가 하락했다는 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>Torm 지분을 19.85%로 확대한 이후 주가 하락 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S19" t="inlineStr">
@@ -1625,7 +1615,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 소형 가전 및 특수 가정용 기기를 설계·판매·유통한다.</ns0:t>
+          <ns0:t>미국과 해외에서 소형 가전 및 특수 가정용 기기를 설계·판매·유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1667,7 +1657,7 @@
       </ns0:c>
       <ns0:c r="R20" t="inlineStr">
         <ns0:is>
-          <ns0:t>동종업체 대비 주가 성과와 저평가 소비재 종목으로서의 투자 매력을 검토한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>동종 기업 대비 주가 성과 우위와 저렴한 소비재 종목으로서의 매수 적합성을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S20" t="inlineStr">
@@ -1709,7 +1699,7 @@
       </ns0:c>
       <ns0:c r="F21" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국과 해외에서 다양한 형태의 맞춤형 냉간 성형 강재를 제조·판매하는 회사.</ns0:t>
+          <ns0:t>중국과 해외에서 다양한 맞춤형 냉간 성형 강재를 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G21">
@@ -1788,7 +1778,7 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술로 의료 제공을 자동화하며 급성 부상·만성 통증·수술 후 재활 등 근골격계 관리 플랫폼을 개발한다.</ns0:t>
+          <ns0:t>기술로 의료 제공을 자동화하며 급성 부상·만성 통증·수술 후 재활 등 근골격계 관리 플랫폼 개발.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22">
@@ -1872,7 +1862,7 @@
       </ns0:c>
       <ns0:c r="F23" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 통신·결제 서비스를 제공하며 소매 솔루션, 핀테크, 인터넷 전화 사업을 운영한다.</ns0:t>
+          <ns0:t>미국·영국 등에서 통신·결제 서비스를 제공하며 소매 솔루션·핀테크·인터넷 전화 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G23">
@@ -1914,7 +1904,7 @@
       </ns0:c>
       <ns0:c r="R23" t="inlineStr">
         <ns0:is>
-          <ns0:t>주가 급등을 다룬 기사와 2026년 4분기 실적 발표 콘퍼런스콜 요약·전문. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>주가 급등 배경을 다룬 기사와 2026년 4분기 실적 발표 콘퍼런스콜 요약·전문. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S23" t="inlineStr">
@@ -1956,7 +1946,7 @@
       </ns0:c>
       <ns0:c r="F24" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 유전·유전체 분석용 시퀀싱 및 어레이 기반 장비와 시약 등 소모품을 제공한다.</ns0:t>
+          <ns0:t>전 세계에 유전·유전체 분석용 시퀀싱·어레이 장비와 시약 등 소모품을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24">
@@ -1998,7 +1988,7 @@
       </ns0:c>
       <ns0:c r="R24" t="inlineStr">
         <ns0:is>
-          <ns0:t>매도 논거와 대체 종목, REGN 대비 가치평가, 옵션시장의 주가 급등 예측 가능성을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>매도 논거와 REGN 대비 가치평가 비교, 옵션시장의 주가 급등 예측 가능성을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S24" t="inlineStr">
@@ -2040,7 +2030,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유와 석유제품의 국제 운송을 위한 원양 선박을 보유·운영하는 기업.</ns0:t>
+          <ns0:t>원유·석유제품의 국제 운송용 원양 선박을 보유·운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2082,7 +2072,7 @@
       </ns0:c>
       <ns0:c r="R25" t="inlineStr">
         <ns0:is>
-          <ns0:t>운송 차질에 따른 기록적 유조선 이익이 낙관론에 미칠 영향과 배당을 분석한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>운송 차질 속 기록적 탱커 이익이 낙관론에 미칠 영향과 배당 분석을 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S25" t="inlineStr">
@@ -2124,7 +2114,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2200,7 +2190,7 @@
       </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
-          <ns0:t>망막 질환 치료제를 연구·개발·상용화하는 임상 단계 바이오제약사로 주요 후보는 타르코시맙 테드로머.</ns0:t>
+          <ns0:t>망막 질환 치료제를 개발·상용화하는 임상 단계 바이오제약사. 주요 후보는 타르코시맙 테드로머.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G27">
@@ -2242,7 +2232,7 @@
       </ns0:c>
       <ns0:c r="R27" t="inlineStr">
         <ns0:is>
-          <ns0:t>긍정적인 습성 황반변성 데이터와 BLA 제출 임박 소식, 주가 178% 상승 및 52주 신고가 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>긍정적 습성 황반변성 데이터와 생물학적제제 허가신청 임박, 주가 급등 및 52주 신고가를 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S27" t="inlineStr">
@@ -2284,7 +2274,7 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28">
@@ -2360,7 +2350,7 @@
       </ns0:c>
       <ns0:c r="F29" t="inlineStr">
         <ns0:is>
-          <ns0:t>보건·안전 분야에 사용하는 휴대용 질량분석기와 푸리에 변환 적외선 장비를 제공한다.</ns0:t>
+          <ns0:t>보건·안전 분야용 휴대용 질량분석기와 푸리에 변환 적외선 장비 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29">
@@ -2439,7 +2429,7 @@
       </ns0:c>
       <ns0:c r="F30" t="inlineStr">
         <ns0:is>
-          <ns0:t>미주·유럽·아시아 등 전 세계에서 실험실 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
+          <ns0:t>전 세계에서 실험실 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G30">
@@ -2481,7 +2471,7 @@
       </ns0:c>
       <ns0:c r="R30" t="inlineStr">
         <ns0:is>
-          <ns0:t>메틀러톨레도가 새롭게 주목받는 배경을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>메틀러토레도가 새롭게 주목받는 배경을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S30" t="inlineStr">
@@ -2523,7 +2513,7 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>일리노이주에서 당좌·저축·정기예금 등 은행 서비스를 제공하는 North Shore Trust and Savings의 지주회사.</ns0:t>
+          <ns0:t>일리노이주에서 당좌·저축·정기예금을 제공하는 North Shore Trust and Savings의 지주사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31">
@@ -2602,7 +2592,7 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계 기업의 데이터 인프라 전환을 위한 소프트웨어·시스템·서비스를 제공한다.</ns0:t>
+          <ns0:t>기업의 데이터 인프라 전환을 위한 소프트웨어·시스템·서비스를 전 세계에 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32">
@@ -2644,7 +2634,7 @@
       </ns0:c>
       <ns0:c r="R32" t="inlineStr">
         <ns0:is>
-          <ns0:t>유럽 규제 데이터 시장 공략과 AI 제휴 확대를 다뤘으며, BofA는 AI 성장 기회를 평가해 목표가를 상향. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>유럽 규제 데이터 시장 공략, AI 성장 기회에 대한 BofA 목표가 상향, 제휴를 통한 AI 전략 확대. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S32" t="inlineStr">
@@ -2686,7 +2676,7 @@
       </ns0:c>
       <ns0:c r="F33" t="inlineStr">
         <ns0:is>
-          <ns0:t>분자검사 서비스를 개발·상용화하며 잔존질환 평가·재발 감시·치료 반응 평가용 혈액검사를 제공한다.</ns0:t>
+          <ns0:t>분자검사를 개발·상용화하며 잔존질환·재발 감시·치료 반응 평가용 혈액검사를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G33">
@@ -2728,7 +2718,7 @@
       </ns0:c>
       <ns0:c r="R33" t="inlineStr">
         <ns0:is>
-          <ns0:t>시그나테라의 방광암 동반진단 일본 PMDA 승인과 주가 급등이 보도됐다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>시그나테라가 일본 PMDA의 방광암 동반진단 승인을 받았으며, 주가 급등을 다룬 기사도 나왔다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S33" t="inlineStr">
@@ -2770,7 +2760,7 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 소비재·기술 분야 기업과의 합병·인수 등 사업결합을 추진하는 기업.</ns0:t>
+          <ns0:t>주요 영업활동 없이 소비재·기술 기업과의 합병·인수 등 사업결합을 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34">
@@ -2846,7 +2836,7 @@
       </ns0:c>
       <ns0:c r="F35" t="inlineStr">
         <ns0:is>
-          <ns0:t>북미와 독일에서 상업·산업·정부용 에너지 관리 시스템을 연구·설계·제조·판매·설치한다.</ns0:t>
+          <ns0:t>북미·독일에서 상업·산업·정부용 에너지 관리 시스템을 연구·설계·제조·판매·설치한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G35">
@@ -2888,7 +2878,7 @@
       </ns0:c>
       <ns0:c r="R35" t="inlineStr">
         <ns0:is>
-          <ns0:t>실적 전망 상향과 소매업체 대상 사업 기회의 확실성을 점검하는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>실적 전망 상향과 소매업체 관련 사업 기회의 확실성을 점검한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S35" t="inlineStr">
@@ -2930,7 +2920,7 @@
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>데이터 저장·관리 기술과 제품을 제공하며 Purity 소프트웨어로 데이터 축소·보호·암호화를 지원한다.</ns0:t>
+          <ns0:t>데이터 저장·관리 제품을 제공하며 Purity 소프트웨어로 데이터 축소·보호·암호화를 지원.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36">
@@ -2972,7 +2962,7 @@
       </ns0:c>
       <ns0:c r="R36" t="inlineStr">
         <ns0:is>
-          <ns0:t>4배 상승 후 저평가 가능성, AI 플랫폼 개선, 애널리스트 목표가 상향과 잉여현금흐름 적자 전환을 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>주가 4배 상승 후 저평가 가능성, AI 플랫폼 개선, 분석가 목표가 상향과 잉여현금흐름 적자를 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S36" t="inlineStr">
@@ -3014,7 +3004,7 @@
       </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 사이버보안 솔루션을 제공하며 보안 접속과 네트워크 보안 관리 제품을 운영하는 기업.</ns0:t>
+          <ns0:t>전 세계에 사이버보안 솔루션과 보안 접속·네트워크 보안 관리 제품을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G37">
@@ -3056,7 +3046,7 @@
       </ns0:c>
       <ns0:c r="R37" t="inlineStr">
         <ns0:is>
-          <ns0:t>AI 방어의 상시 서비스화와 주가 상승 보도, 크라우드스트라이크와의 투자 비교 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>AI 방어의 상시 서비스화와 주가 상승 동향, 크라우드스트라이크와의 투자 비교를 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S37" t="inlineStr">
@@ -3098,7 +3088,7 @@
       </ns0:c>
       <ns0:c r="F38" t="inlineStr">
         <ns0:is>
-          <ns0:t>암 치료 제품을 개발·상용화하는 바이오제약사로, 경구용 네라티닙 제품 NERLYNX를 제공.</ns0:t>
+          <ns0:t>암 치료제를 개발·상용화하며 경구용 네라티닙 제품 NERLYNX를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G38">
@@ -3182,7 +3172,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>정밀 기술을 활용해 면역항암·자가면역·감염 질환 대상 유전자·세포 치료제를 개발.</ns0:t>
+          <ns0:t>정밀 기술을 활용해 면역항암·자가면역·감염 질환용 유전자·세포 치료제를 개발.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3224,7 +3214,7 @@
       </ns0:c>
       <ns0:c r="R39" t="inlineStr">
         <ns0:is>
-          <ns0:t>FDA의 플랫폼 인정과 신약 개발비 절감 가능성, 기업가치 평가 및 수년 내 주가 최고치 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>FDA의 플랫폼 인정과 신약 개발비 절감 가능성, 저평가 여부 및 다년 신고가 동향을 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S39" t="inlineStr">
@@ -3266,7 +3256,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·클라우드·SaaS 데이터 보호, 위협 분석 및 신원 복구 등 데이터 보안 솔루션 제공.</ns0:t>
+          <ns0:t>기업·클라우드·SaaS 데이터 보호, 위협 분석, 신원 복구 등 데이터 보안 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3350,7 +3340,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 독자 기술과 분석 역량으로 신원 정보 및 조사 솔루션 idiCORE를 제공.</ns0:t>
+          <ns0:t>미국에서 독자 기술과 분석 역량을 활용한 신원 정보·조사 솔루션 idiCORE를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3392,7 +3382,7 @@
       </ns0:c>
       <ns0:c r="R41" t="inlineStr">
         <ns0:is>
-          <ns0:t>높은 주가수익비율과 주가 모멘텀 속에서도 6% 저평가 가능성 제기. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>높은 주가수익비율과 주가 모멘텀 속에서도 6% 저평가됐을 가능성을 제시. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S41" t="inlineStr">
@@ -3434,7 +3424,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>보건과학 분야의 장비·시약·소프트웨어·검사 플랫폼과 탐지·영상 기술 및 서비스를 제공한다.</ns0:t>
+          <ns0:t>보건과학용 장비·시약·소프트웨어·검사 플랫폼과 탐지·영상 기술 및 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3476,7 +3466,7 @@
       </ns0:c>
       <ns0:c r="R42" t="inlineStr">
         <ns0:is>
-          <ns0:t>2분기 실적 후 투자 판단과 보유 논거, 유럽 신생아 1형 당뇨병 탐지 키트 출시를 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>2분기 실적 후 투자 판단과 보유 논거, 유럽 내 신생아 제1형 당뇨병 탐지 키트 출시를 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S42" t="inlineStr">
@@ -3518,7 +3508,7 @@
       </ns0:c>
       <ns0:c r="F43" t="inlineStr">
         <ns0:is>
-          <ns0:t>신약 개발과 소재 응용을 위한 신규 분자 발굴용 물리학 기반 계산 플랫폼을 개발.</ns0:t>
+          <ns0:t>신약 개발·소재 응용을 위한 신규 분자 발굴용 물리학 기반 계산 플랫폼을 개발.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G43">
@@ -3602,7 +3592,7 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>서버 네트워크 인터페이스 카드와 암호화·압축용 카드 등 네트워크·데이터 인프라 솔루션을 설계·제조·판매.</ns0:t>
+          <ns0:t>서버 네트워크 인터페이스 카드와 암호화·압축용 카드 등 네트워크·데이터 인프라 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44">
@@ -3839,7 +3829,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 생명과학 솔루션, 분석기기, 전문 진단, 실험실 제품 및 바이오제약 서비스를 제공.</ns0:t>
+          <ns0:t>전 세계에 생명과학 솔루션·분석기기·전문 진단·실험실 제품·바이오제약 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">
@@ -3881,7 +3871,7 @@
       </ns0:c>
       <ns0:c r="R47" t="inlineStr">
         <ns0:is>
-          <ns0:t>47% 상승 후 주가 적정성 평가, 혁신의 반복매출 전환과 수익성, 신규 CHO-K1 패널·MRD 행보 조명. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>47% 상승 후 가치평가, 혁신의 반복 매출 전환과 수익성, 신규 CHO-K1 패널·MRD 행보를 다룸. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S47" t="inlineStr">
@@ -3923,7 +3913,7 @@
       </ns0:c>
       <ns0:c r="F48" t="inlineStr">
         <ns0:is>
-          <ns0:t>석유제품 운반선을 보유·운영하며 휘발유·항공유 등 정제유 운송과 해양 엔지니어링 사업을 영위.</ns0:t>
+          <ns0:t>석유제품 운반선을 보유·운영하며 정제유 운송과 해양 엔지니어링 사업을 영위.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G48">
@@ -3965,7 +3955,7 @@
       </ns0:c>
       <ns0:c r="R48" t="inlineStr">
         <ns0:is>
-          <ns0:t>하프니아가 TORM 지분을 19.85%로 늘린 뒤 하프니아 주가 하락 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>하프니아가 Torm 지분을 19.85%로 늘린 뒤 하프니아 주가가 하락했다는 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S48" t="inlineStr">
@@ -4007,7 +3997,7 @@
       </ns0:c>
       <ns0:c r="F49" t="inlineStr">
         <ns0:is>
-          <ns0:t>치료제·진단·소재·식품·농업·데이터 저장·학술 연구 등에 쓰이는 합성 DNA 제품을 제조·판매한다.</ns0:t>
+          <ns0:t>치료제·진단·소재·식품·농업·데이터 저장·학술 연구용 합성 DNA 제품을 제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G49">
@@ -4049,7 +4039,7 @@
       </ns0:c>
       <ns0:c r="R49" t="inlineStr">
         <ns0:is>
-          <ns0:t>매수에 필요한 조건을 검토한 기사와 목요일 주가 16% 상승을 앤트로픽과 연관 지은 리링크의 평가. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>매수 판단 조건을 다룬 기사와 목요일 주가 16% 상승을 앤트로픽과 연결한 리링크의 해석 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S49" t="inlineStr">
@@ -4091,7 +4081,7 @@
       </ns0:c>
       <ns0:c r="F50" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 생물학적 시스템 분석용 장비·소모품·소프트웨어를 개발·판매하며 Chromium 플랫폼을 제공한다.</ns0:t>
+          <ns0:t>생물학적 시스템 분석용 장비·소모품·소프트웨어를 개발·판매하며 Chromium 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G50">
@@ -4133,7 +4123,7 @@
       </ns0:c>
       <ns0:c r="R50" t="inlineStr">
         <ns0:is>
-          <ns0:t>10x 지노믹스의 주가 상승을 다룬 기사와 여러 의료 관련 종목의 동반 하락을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>10x Genomics 주가 상승 보도와 여러 의료 관련 종목과 함께 하락했다는 보도가 각각 제시됨. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S50" t="inlineStr">
@@ -4175,7 +4165,7 @@
       </ns0:c>
       <ns0:c r="F51" t="inlineStr">
         <ns0:is>
-          <ns0:t>파키스탄·우크라이나·카자흐스탄·방글라데시·우즈베키스탄에서 통신·디지털 서비스를 제공.</ns0:t>
+          <ns0:t>파키스탄·우크라이나·카자흐스탄·방글라데시·우즈베키스탄에서 통신·디지털 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G51">
@@ -4217,7 +4207,7 @@
       </ns0:c>
       <ns0:c r="R51" t="inlineStr">
         <ns0:is>
-          <ns0:t>방글라데시 디지털은행 면허 취득과 기업가치 평가 논쟁 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>기업가치 평가 논쟁이 커지는 가운데 방글라데시 디지털 은행 면허를 취득했다는 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S51" t="inlineStr">
@@ -4335,7 +4325,7 @@
       </ns0:c>
       <ns0:c r="F53" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 여성 핸드백, 여행가방·용품, 패션·홈 액세서리 및 선물용품을 설계·제조.</ns0:t>
+          <ns0:t>미국에서 여성 핸드백, 여행가방·용품, 패션·홈 액세서리와 선물용품을 설계·제조.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G53">
@@ -4377,7 +4367,7 @@
       </ns0:c>
       <ns0:c r="R53" t="inlineStr">
         <ns0:is>
-          <ns0:t>빠른 주가 움직임을 보이는 베라 브래들리의 가치투자 매력을 평가한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>빠른 주가 움직임을 보인 Vera Bradley의 가치투자 매력을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S53" t="inlineStr">
@@ -4419,7 +4409,7 @@
       </ns0:c>
       <ns0:c r="F54" t="inlineStr">
         <ns0:is>
-          <ns0:t>아시아·미주·유럽에서 분석 업무 솔루션과 액체크로마토그래피·질량분석 시스템을 제공.</ns0:t>
+          <ns0:t>아시아·미주·유럽에서 분석 업무 솔루션과 액체크로마토그래피·질량분석 시스템 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G54">
@@ -4461,7 +4451,7 @@
       </ns0:c>
       <ns0:c r="R54" t="inlineStr">
         <ns0:is>
-          <ns0:t>가정용 HPV 검사·세포 분석 진출이 낙관론에 미칠 영향과 성장 전망 상회, AI 수요·BD 통합 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>가정용 HPV·세포 분석 추진이 낙관론에 미칠 영향과 AI 수요·BD 통합 속 성장 전망 상회 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S54" t="inlineStr">
@@ -4503,7 +4493,7 @@
       </ns0:c>
       <ns0:c r="F55" t="inlineStr">
         <ns0:is>
-          <ns0:t>HBO Max·discovery+ 등 스트리밍, 스튜디오 및 글로벌 방송 네트워크를 운영하는 미디어 기업.</ns0:t>
+          <ns0:t>HBO Max·discovery+ 등 스트리밍, 스튜디오와 글로벌 방송 네트워크를 운영하는 미디어 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G55">
@@ -4666,7 +4656,7 @@
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>유의미한 영업활동 없이 기업 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
+          <ns0:t>유의미한 영업활동 없이 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57">
@@ -4718,102 +4708,101 @@
   <ns0:autoFilter ref="A1:T57"/>
   <ns0:hyperlinks>
     <ns0:hyperlink ref="S2" ns1:id="rId1"/>
-    <ns0:hyperlink ref="T2" ns1:id="rId2"/>
-    <ns0:hyperlink ref="S3" ns1:id="rId3"/>
-    <ns0:hyperlink ref="T3" ns1:id="rId4"/>
-    <ns0:hyperlink ref="T4" ns1:id="rId5"/>
-    <ns0:hyperlink ref="S5" ns1:id="rId6"/>
-    <ns0:hyperlink ref="T5" ns1:id="rId7"/>
-    <ns0:hyperlink ref="S6" ns1:id="rId8"/>
-    <ns0:hyperlink ref="T6" ns1:id="rId9"/>
-    <ns0:hyperlink ref="S7" ns1:id="rId10"/>
-    <ns0:hyperlink ref="T7" ns1:id="rId11"/>
-    <ns0:hyperlink ref="S8" ns1:id="rId12"/>
-    <ns0:hyperlink ref="T8" ns1:id="rId13"/>
-    <ns0:hyperlink ref="S9" ns1:id="rId14"/>
-    <ns0:hyperlink ref="T9" ns1:id="rId15"/>
-    <ns0:hyperlink ref="S10" ns1:id="rId16"/>
-    <ns0:hyperlink ref="T10" ns1:id="rId17"/>
-    <ns0:hyperlink ref="S11" ns1:id="rId18"/>
-    <ns0:hyperlink ref="T11" ns1:id="rId19"/>
-    <ns0:hyperlink ref="S12" ns1:id="rId20"/>
-    <ns0:hyperlink ref="T12" ns1:id="rId21"/>
-    <ns0:hyperlink ref="S13" ns1:id="rId22"/>
-    <ns0:hyperlink ref="T13" ns1:id="rId23"/>
-    <ns0:hyperlink ref="T14" ns1:id="rId24"/>
-    <ns0:hyperlink ref="T15" ns1:id="rId25"/>
-    <ns0:hyperlink ref="S16" ns1:id="rId26"/>
-    <ns0:hyperlink ref="T16" ns1:id="rId27"/>
-    <ns0:hyperlink ref="S17" ns1:id="rId28"/>
-    <ns0:hyperlink ref="T17" ns1:id="rId29"/>
-    <ns0:hyperlink ref="S18" ns1:id="rId30"/>
-    <ns0:hyperlink ref="T18" ns1:id="rId31"/>
-    <ns0:hyperlink ref="S19" ns1:id="rId32"/>
-    <ns0:hyperlink ref="T19" ns1:id="rId33"/>
-    <ns0:hyperlink ref="S20" ns1:id="rId34"/>
-    <ns0:hyperlink ref="T20" ns1:id="rId35"/>
-    <ns0:hyperlink ref="T21" ns1:id="rId36"/>
-    <ns0:hyperlink ref="S22" ns1:id="rId37"/>
-    <ns0:hyperlink ref="T22" ns1:id="rId38"/>
-    <ns0:hyperlink ref="S23" ns1:id="rId39"/>
-    <ns0:hyperlink ref="T23" ns1:id="rId40"/>
-    <ns0:hyperlink ref="S24" ns1:id="rId41"/>
-    <ns0:hyperlink ref="T24" ns1:id="rId42"/>
-    <ns0:hyperlink ref="S25" ns1:id="rId43"/>
-    <ns0:hyperlink ref="T25" ns1:id="rId44"/>
-    <ns0:hyperlink ref="T26" ns1:id="rId45"/>
-    <ns0:hyperlink ref="S27" ns1:id="rId46"/>
-    <ns0:hyperlink ref="T27" ns1:id="rId47"/>
-    <ns0:hyperlink ref="T28" ns1:id="rId48"/>
-    <ns0:hyperlink ref="T29" ns1:id="rId49"/>
-    <ns0:hyperlink ref="S30" ns1:id="rId50"/>
-    <ns0:hyperlink ref="T30" ns1:id="rId51"/>
-    <ns0:hyperlink ref="T31" ns1:id="rId52"/>
-    <ns0:hyperlink ref="S32" ns1:id="rId53"/>
-    <ns0:hyperlink ref="T32" ns1:id="rId54"/>
-    <ns0:hyperlink ref="S33" ns1:id="rId55"/>
-    <ns0:hyperlink ref="T33" ns1:id="rId56"/>
-    <ns0:hyperlink ref="T34" ns1:id="rId57"/>
-    <ns0:hyperlink ref="S35" ns1:id="rId58"/>
-    <ns0:hyperlink ref="T35" ns1:id="rId59"/>
-    <ns0:hyperlink ref="S36" ns1:id="rId60"/>
-    <ns0:hyperlink ref="T36" ns1:id="rId61"/>
-    <ns0:hyperlink ref="S37" ns1:id="rId62"/>
-    <ns0:hyperlink ref="T37" ns1:id="rId63"/>
-    <ns0:hyperlink ref="S38" ns1:id="rId64"/>
-    <ns0:hyperlink ref="T38" ns1:id="rId65"/>
-    <ns0:hyperlink ref="S39" ns1:id="rId66"/>
-    <ns0:hyperlink ref="T39" ns1:id="rId67"/>
-    <ns0:hyperlink ref="S40" ns1:id="rId68"/>
-    <ns0:hyperlink ref="T40" ns1:id="rId69"/>
-    <ns0:hyperlink ref="S41" ns1:id="rId70"/>
-    <ns0:hyperlink ref="T41" ns1:id="rId71"/>
-    <ns0:hyperlink ref="S42" ns1:id="rId72"/>
-    <ns0:hyperlink ref="T42" ns1:id="rId73"/>
-    <ns0:hyperlink ref="S43" ns1:id="rId74"/>
-    <ns0:hyperlink ref="T43" ns1:id="rId75"/>
-    <ns0:hyperlink ref="T44" ns1:id="rId76"/>
-    <ns0:hyperlink ref="T45" ns1:id="rId77"/>
-    <ns0:hyperlink ref="T46" ns1:id="rId78"/>
-    <ns0:hyperlink ref="S47" ns1:id="rId79"/>
-    <ns0:hyperlink ref="T47" ns1:id="rId80"/>
-    <ns0:hyperlink ref="S48" ns1:id="rId81"/>
-    <ns0:hyperlink ref="T48" ns1:id="rId82"/>
-    <ns0:hyperlink ref="S49" ns1:id="rId83"/>
-    <ns0:hyperlink ref="T49" ns1:id="rId84"/>
-    <ns0:hyperlink ref="S50" ns1:id="rId85"/>
-    <ns0:hyperlink ref="T50" ns1:id="rId86"/>
-    <ns0:hyperlink ref="S51" ns1:id="rId87"/>
-    <ns0:hyperlink ref="T51" ns1:id="rId88"/>
-    <ns0:hyperlink ref="T52" ns1:id="rId89"/>
-    <ns0:hyperlink ref="S53" ns1:id="rId90"/>
-    <ns0:hyperlink ref="T53" ns1:id="rId91"/>
-    <ns0:hyperlink ref="S54" ns1:id="rId92"/>
-    <ns0:hyperlink ref="T54" ns1:id="rId93"/>
-    <ns0:hyperlink ref="S55" ns1:id="rId94"/>
-    <ns0:hyperlink ref="T55" ns1:id="rId95"/>
-    <ns0:hyperlink ref="T56" ns1:id="rId96"/>
-    <ns0:hyperlink ref="T57" ns1:id="rId97"/>
+    <ns0:hyperlink ref="S3" ns1:id="rId2"/>
+    <ns0:hyperlink ref="T3" ns1:id="rId3"/>
+    <ns0:hyperlink ref="T4" ns1:id="rId4"/>
+    <ns0:hyperlink ref="S5" ns1:id="rId5"/>
+    <ns0:hyperlink ref="T5" ns1:id="rId6"/>
+    <ns0:hyperlink ref="S6" ns1:id="rId7"/>
+    <ns0:hyperlink ref="T6" ns1:id="rId8"/>
+    <ns0:hyperlink ref="S7" ns1:id="rId9"/>
+    <ns0:hyperlink ref="T7" ns1:id="rId10"/>
+    <ns0:hyperlink ref="S8" ns1:id="rId11"/>
+    <ns0:hyperlink ref="T8" ns1:id="rId12"/>
+    <ns0:hyperlink ref="S9" ns1:id="rId13"/>
+    <ns0:hyperlink ref="T9" ns1:id="rId14"/>
+    <ns0:hyperlink ref="S10" ns1:id="rId15"/>
+    <ns0:hyperlink ref="T10" ns1:id="rId16"/>
+    <ns0:hyperlink ref="S11" ns1:id="rId17"/>
+    <ns0:hyperlink ref="T11" ns1:id="rId18"/>
+    <ns0:hyperlink ref="S12" ns1:id="rId19"/>
+    <ns0:hyperlink ref="T12" ns1:id="rId20"/>
+    <ns0:hyperlink ref="S13" ns1:id="rId21"/>
+    <ns0:hyperlink ref="T13" ns1:id="rId22"/>
+    <ns0:hyperlink ref="T14" ns1:id="rId23"/>
+    <ns0:hyperlink ref="T15" ns1:id="rId24"/>
+    <ns0:hyperlink ref="S16" ns1:id="rId25"/>
+    <ns0:hyperlink ref="T16" ns1:id="rId26"/>
+    <ns0:hyperlink ref="S17" ns1:id="rId27"/>
+    <ns0:hyperlink ref="T17" ns1:id="rId28"/>
+    <ns0:hyperlink ref="S18" ns1:id="rId29"/>
+    <ns0:hyperlink ref="T18" ns1:id="rId30"/>
+    <ns0:hyperlink ref="S19" ns1:id="rId31"/>
+    <ns0:hyperlink ref="T19" ns1:id="rId32"/>
+    <ns0:hyperlink ref="S20" ns1:id="rId33"/>
+    <ns0:hyperlink ref="T20" ns1:id="rId34"/>
+    <ns0:hyperlink ref="T21" ns1:id="rId35"/>
+    <ns0:hyperlink ref="S22" ns1:id="rId36"/>
+    <ns0:hyperlink ref="T22" ns1:id="rId37"/>
+    <ns0:hyperlink ref="S23" ns1:id="rId38"/>
+    <ns0:hyperlink ref="T23" ns1:id="rId39"/>
+    <ns0:hyperlink ref="S24" ns1:id="rId40"/>
+    <ns0:hyperlink ref="T24" ns1:id="rId41"/>
+    <ns0:hyperlink ref="S25" ns1:id="rId42"/>
+    <ns0:hyperlink ref="T25" ns1:id="rId43"/>
+    <ns0:hyperlink ref="T26" ns1:id="rId44"/>
+    <ns0:hyperlink ref="S27" ns1:id="rId45"/>
+    <ns0:hyperlink ref="T27" ns1:id="rId46"/>
+    <ns0:hyperlink ref="T28" ns1:id="rId47"/>
+    <ns0:hyperlink ref="T29" ns1:id="rId48"/>
+    <ns0:hyperlink ref="S30" ns1:id="rId49"/>
+    <ns0:hyperlink ref="T30" ns1:id="rId50"/>
+    <ns0:hyperlink ref="T31" ns1:id="rId51"/>
+    <ns0:hyperlink ref="S32" ns1:id="rId52"/>
+    <ns0:hyperlink ref="T32" ns1:id="rId53"/>
+    <ns0:hyperlink ref="S33" ns1:id="rId54"/>
+    <ns0:hyperlink ref="T33" ns1:id="rId55"/>
+    <ns0:hyperlink ref="T34" ns1:id="rId56"/>
+    <ns0:hyperlink ref="S35" ns1:id="rId57"/>
+    <ns0:hyperlink ref="T35" ns1:id="rId58"/>
+    <ns0:hyperlink ref="S36" ns1:id="rId59"/>
+    <ns0:hyperlink ref="T36" ns1:id="rId60"/>
+    <ns0:hyperlink ref="S37" ns1:id="rId61"/>
+    <ns0:hyperlink ref="T37" ns1:id="rId62"/>
+    <ns0:hyperlink ref="S38" ns1:id="rId63"/>
+    <ns0:hyperlink ref="T38" ns1:id="rId64"/>
+    <ns0:hyperlink ref="S39" ns1:id="rId65"/>
+    <ns0:hyperlink ref="T39" ns1:id="rId66"/>
+    <ns0:hyperlink ref="S40" ns1:id="rId67"/>
+    <ns0:hyperlink ref="T40" ns1:id="rId68"/>
+    <ns0:hyperlink ref="S41" ns1:id="rId69"/>
+    <ns0:hyperlink ref="T41" ns1:id="rId70"/>
+    <ns0:hyperlink ref="S42" ns1:id="rId71"/>
+    <ns0:hyperlink ref="T42" ns1:id="rId72"/>
+    <ns0:hyperlink ref="S43" ns1:id="rId73"/>
+    <ns0:hyperlink ref="T43" ns1:id="rId74"/>
+    <ns0:hyperlink ref="T44" ns1:id="rId75"/>
+    <ns0:hyperlink ref="T45" ns1:id="rId76"/>
+    <ns0:hyperlink ref="T46" ns1:id="rId77"/>
+    <ns0:hyperlink ref="S47" ns1:id="rId78"/>
+    <ns0:hyperlink ref="T47" ns1:id="rId79"/>
+    <ns0:hyperlink ref="S48" ns1:id="rId80"/>
+    <ns0:hyperlink ref="T48" ns1:id="rId81"/>
+    <ns0:hyperlink ref="S49" ns1:id="rId82"/>
+    <ns0:hyperlink ref="T49" ns1:id="rId83"/>
+    <ns0:hyperlink ref="S50" ns1:id="rId84"/>
+    <ns0:hyperlink ref="T50" ns1:id="rId85"/>
+    <ns0:hyperlink ref="S51" ns1:id="rId86"/>
+    <ns0:hyperlink ref="T51" ns1:id="rId87"/>
+    <ns0:hyperlink ref="T52" ns1:id="rId88"/>
+    <ns0:hyperlink ref="S53" ns1:id="rId89"/>
+    <ns0:hyperlink ref="T53" ns1:id="rId90"/>
+    <ns0:hyperlink ref="S54" ns1:id="rId91"/>
+    <ns0:hyperlink ref="T54" ns1:id="rId92"/>
+    <ns0:hyperlink ref="S55" ns1:id="rId93"/>
+    <ns0:hyperlink ref="T55" ns1:id="rId94"/>
+    <ns0:hyperlink ref="T56" ns1:id="rId95"/>
+    <ns0:hyperlink ref="T57" ns1:id="rId96"/>
   </ns0:hyperlinks>
 </ns0:worksheet>
 </file>

</xml_diff>